<commit_message>
Load three scaled source files, including renewal, SEM, Facebook, and content metrics.
</commit_message>
<xml_diff>
--- a/public/samples/ctia-social-monthly.xlsx
+++ b/public/samples/ctia-social-monthly.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
@@ -452,34 +452,34 @@
         <v>-發送篇數</v>
       </c>
       <c r="B3">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="C3">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>74</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>87</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -487,34 +487,34 @@
         <v>-關注人數</v>
       </c>
       <c r="B4">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C4">
+        <v>15</v>
+      </c>
+      <c r="D4">
+        <v>22</v>
+      </c>
+      <c r="E4">
+        <v>22</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>9</v>
+      </c>
+      <c r="H4">
         <v>17</v>
       </c>
-      <c r="D4">
-        <v>103</v>
-      </c>
-      <c r="E4">
-        <v>116</v>
-      </c>
-      <c r="F4">
-        <v>39</v>
-      </c>
-      <c r="G4">
-        <v>52</v>
-      </c>
-      <c r="H4">
-        <v>65</v>
-      </c>
       <c r="I4">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="J4">
-        <v>181</v>
+        <v>20</v>
       </c>
       <c r="K4">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -522,34 +522,34 @@
         <v>-閱讀/觀看量</v>
       </c>
       <c r="B5">
-        <v>10910</v>
+        <v>8975</v>
       </c>
       <c r="C5">
-        <v>107</v>
+        <v>404</v>
       </c>
       <c r="D5">
-        <v>120</v>
+        <v>1285</v>
       </c>
       <c r="E5">
-        <v>133</v>
+        <v>1580</v>
       </c>
       <c r="F5">
-        <v>146</v>
+        <v>1449</v>
       </c>
       <c r="G5">
-        <v>159</v>
+        <v>1695</v>
       </c>
       <c r="H5">
-        <v>172</v>
+        <v>785</v>
       </c>
       <c r="I5">
-        <v>185</v>
+        <v>1265</v>
       </c>
       <c r="J5">
-        <v>101</v>
+        <v>478</v>
       </c>
       <c r="K5">
-        <v>114</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
@@ -557,34 +557,34 @@
         <v>-喜歡/點讚量</v>
       </c>
       <c r="B6">
-        <v>111</v>
+        <v>1354</v>
       </c>
       <c r="C6">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="D6">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="E6">
-        <v>150</v>
+        <v>325</v>
       </c>
       <c r="F6">
-        <v>163</v>
+        <v>47</v>
       </c>
       <c r="G6">
-        <v>176</v>
+        <v>93</v>
       </c>
       <c r="H6">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I6">
-        <v>105</v>
+        <v>248</v>
       </c>
       <c r="J6">
-        <v>118</v>
+        <v>194</v>
       </c>
       <c r="K6">
-        <v>41</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -592,34 +592,34 @@
         <v>-收藏/推薦量</v>
       </c>
       <c r="B7">
-        <v>128</v>
+        <v>599</v>
       </c>
       <c r="C7">
-        <v>141</v>
+        <v>53</v>
       </c>
       <c r="D7">
-        <v>154</v>
+        <v>76</v>
       </c>
       <c r="E7">
-        <v>167</v>
+        <v>117</v>
       </c>
       <c r="F7">
-        <v>180</v>
+        <v>20</v>
       </c>
       <c r="G7">
-        <v>193</v>
+        <v>43</v>
       </c>
       <c r="H7">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="I7">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J7">
-        <v>135</v>
+        <v>84</v>
       </c>
       <c r="K7">
-        <v>58</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -627,34 +627,34 @@
         <v>-分享量</v>
       </c>
       <c r="B8">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="C8">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="D8">
-        <v>171</v>
+        <v>23</v>
       </c>
       <c r="E8">
-        <v>184</v>
+        <v>21</v>
       </c>
       <c r="F8">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G8">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="H8">
-        <v>126</v>
+        <v>25</v>
       </c>
       <c r="I8">
-        <v>139</v>
+        <v>25</v>
       </c>
       <c r="J8">
-        <v>62</v>
+        <v>19</v>
       </c>
       <c r="K8">
-        <v>75</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -667,34 +667,34 @@
         <v>-曝光量</v>
       </c>
       <c r="B10">
-        <v>10790</v>
+        <v>52707</v>
       </c>
       <c r="C10">
-        <v>192</v>
+        <v>1965</v>
       </c>
       <c r="D10">
-        <v>10080</v>
+        <v>4777</v>
       </c>
       <c r="E10">
-        <v>10210</v>
+        <v>7455</v>
       </c>
       <c r="F10">
-        <v>10340</v>
+        <v>11479</v>
       </c>
       <c r="G10">
-        <v>10470</v>
+        <v>8091</v>
       </c>
       <c r="H10">
-        <v>10600</v>
+        <v>8360</v>
       </c>
       <c r="I10">
-        <v>10730</v>
+        <v>5900</v>
       </c>
       <c r="J10">
-        <v>10860</v>
+        <v>4560</v>
       </c>
       <c r="K10">
-        <v>102</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11">
@@ -702,34 +702,34 @@
         <v>-點擊率</v>
       </c>
       <c r="B11">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="C11">
-        <v>0.17</v>
+        <v>0.209</v>
       </c>
       <c r="D11">
+        <v>0.203</v>
+      </c>
+      <c r="E11">
+        <v>0.194</v>
+      </c>
+      <c r="F11">
+        <v>0.1658</v>
+      </c>
+      <c r="G11">
+        <v>0.1541</v>
+      </c>
+      <c r="H11">
+        <v>0.197</v>
+      </c>
+      <c r="I11">
+        <v>0.186</v>
+      </c>
+      <c r="J11">
+        <v>0.188</v>
+      </c>
+      <c r="K11">
         <v>0.1</v>
-      </c>
-      <c r="E11">
-        <v>0.23</v>
-      </c>
-      <c r="F11">
-        <v>0.16</v>
-      </c>
-      <c r="G11">
-        <v>0.09</v>
-      </c>
-      <c r="H11">
-        <v>0.22</v>
-      </c>
-      <c r="I11">
-        <v>0.15</v>
-      </c>
-      <c r="J11">
-        <v>0.11</v>
-      </c>
-      <c r="K11">
-        <v>0.24</v>
       </c>
     </row>
     <row r="12">
@@ -742,34 +742,34 @@
         <v>-發送篇數</v>
       </c>
       <c r="B13">
-        <v>43</v>
+        <v>8</v>
       </c>
       <c r="C13">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="E13">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="F13">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="I13">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="J13">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="K13">
-        <v>63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -777,34 +777,34 @@
         <v>-關注人數</v>
       </c>
       <c r="B14">
-        <v>150</v>
+        <v>57</v>
       </c>
       <c r="C14">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="D14">
-        <v>86</v>
+        <v>1</v>
       </c>
       <c r="E14">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="F14">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G14">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="I14">
-        <v>144</v>
+        <v>26</v>
       </c>
       <c r="J14">
-        <v>67</v>
+        <v>14</v>
       </c>
       <c r="K14">
-        <v>80</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -812,34 +812,34 @@
         <v>-曝光量</v>
       </c>
       <c r="B15">
-        <v>10670</v>
+        <v>4436</v>
       </c>
       <c r="C15">
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="D15">
-        <v>193</v>
+        <v>539</v>
       </c>
       <c r="E15">
-        <v>109</v>
+        <v>674</v>
       </c>
       <c r="F15">
-        <v>122</v>
+        <v>453</v>
       </c>
       <c r="G15">
-        <v>135</v>
+        <v>480</v>
       </c>
       <c r="H15">
-        <v>148</v>
+        <v>400</v>
       </c>
       <c r="I15">
-        <v>161</v>
+        <v>900</v>
       </c>
       <c r="J15">
-        <v>174</v>
+        <v>600</v>
       </c>
       <c r="K15">
-        <v>187</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16">
@@ -847,34 +847,34 @@
         <v>-觀看量</v>
       </c>
       <c r="B16">
-        <v>184</v>
+        <v>1184</v>
       </c>
       <c r="C16">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="D16">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="E16">
-        <v>126</v>
+        <v>168</v>
       </c>
       <c r="F16">
-        <v>139</v>
+        <v>169</v>
       </c>
       <c r="G16">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="H16">
-        <v>165</v>
+        <v>80</v>
       </c>
       <c r="I16">
-        <v>178</v>
+        <v>240</v>
       </c>
       <c r="J16">
-        <v>191</v>
+        <v>160</v>
       </c>
       <c r="K16">
-        <v>107</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17">
@@ -882,34 +882,34 @@
         <v>-點擊率</v>
       </c>
       <c r="B17">
-        <v>0.09</v>
+        <v>0.13336940348978762</v>
       </c>
       <c r="C17">
-        <v>0.22</v>
+        <v>0.14</v>
       </c>
       <c r="D17">
         <v>0.15</v>
       </c>
       <c r="E17">
-        <v>0.08</v>
+        <v>0.13</v>
       </c>
       <c r="F17">
-        <v>0.21</v>
+        <v>0.1543</v>
       </c>
       <c r="G17">
-        <v>0.14</v>
+        <v>0.1188</v>
       </c>
       <c r="H17">
-        <v>0.07</v>
+        <v>0.12</v>
       </c>
       <c r="I17">
-        <v>0.2</v>
+        <v>0.11</v>
       </c>
       <c r="J17">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
       <c r="K17">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="18">
@@ -917,34 +917,34 @@
         <v>-喜歡</v>
       </c>
       <c r="B18">
-        <v>121</v>
+        <v>634</v>
       </c>
       <c r="C18">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="D18">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="E18">
-        <v>160</v>
+        <v>215</v>
       </c>
       <c r="F18">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="G18">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H18">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="I18">
-        <v>115</v>
+        <v>180</v>
       </c>
       <c r="J18">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="K18">
-        <v>51</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19">
@@ -952,34 +952,34 @@
         <v>-收藏</v>
       </c>
       <c r="B19">
-        <v>138</v>
+        <v>264</v>
       </c>
       <c r="C19">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="D19">
-        <v>74</v>
+        <v>6</v>
       </c>
       <c r="E19">
-        <v>177</v>
+        <v>75</v>
       </c>
       <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>5</v>
+      </c>
+      <c r="H19">
         <v>20</v>
       </c>
-      <c r="G19">
-        <v>16</v>
-      </c>
-      <c r="H19">
-        <v>119</v>
-      </c>
       <c r="I19">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="J19">
-        <v>145</v>
+        <v>60</v>
       </c>
       <c r="K19">
-        <v>68</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -987,34 +987,34 @@
         <v>-分享</v>
       </c>
       <c r="B20">
-        <v>155</v>
+        <v>53</v>
       </c>
       <c r="C20">
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="D20">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E20">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F20">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="G20">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="H20">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="I20">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="J20">
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="K20">
-        <v>85</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1027,31 +1027,31 @@
         <v>-發送篇數</v>
       </c>
       <c r="B22">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C22">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E22">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="F22">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="H22">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="I22">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="J22">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -1062,34 +1062,34 @@
         <v>-關注人數</v>
       </c>
       <c r="B23">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="C23">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D23">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="E23">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="F23">
-        <v>71</v>
+        <v>8</v>
       </c>
       <c r="G23">
-        <v>84</v>
+        <v>5</v>
       </c>
       <c r="H23">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="I23">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J23">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="K23">
-        <v>39</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1097,31 +1097,31 @@
         <v>-曝光量</v>
       </c>
       <c r="B24">
-        <v>10260</v>
+        <v>45348</v>
       </c>
       <c r="C24">
-        <v>139</v>
+        <v>1695</v>
       </c>
       <c r="D24">
-        <v>10520</v>
+        <v>4238</v>
       </c>
       <c r="E24">
-        <v>10650</v>
+        <v>6780</v>
       </c>
       <c r="F24">
-        <v>10780</v>
+        <v>11026</v>
       </c>
       <c r="G24">
-        <v>10910</v>
+        <v>7609</v>
       </c>
       <c r="H24">
-        <v>10070</v>
+        <v>6000</v>
       </c>
       <c r="I24">
-        <v>10200</v>
+        <v>5000</v>
       </c>
       <c r="J24">
-        <v>10330</v>
+        <v>3000</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -1132,31 +1132,31 @@
         <v>-觀看量</v>
       </c>
       <c r="B25">
-        <v>10430</v>
+        <v>7211</v>
       </c>
       <c r="C25">
-        <v>156</v>
+        <v>337</v>
       </c>
       <c r="D25">
-        <v>169</v>
+        <v>842</v>
       </c>
       <c r="E25">
-        <v>182</v>
+        <v>1347</v>
       </c>
       <c r="F25">
-        <v>195</v>
+        <v>1281</v>
       </c>
       <c r="G25">
-        <v>111</v>
+        <v>1504</v>
       </c>
       <c r="H25">
-        <v>124</v>
+        <v>600</v>
       </c>
       <c r="I25">
-        <v>137</v>
+        <v>1000</v>
       </c>
       <c r="J25">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -1167,31 +1167,31 @@
         <v>-點擊率</v>
       </c>
       <c r="B26">
-        <v>0.05</v>
+        <v>0.15898476261880085</v>
       </c>
       <c r="C26">
-        <v>0.18</v>
+        <v>0.22</v>
       </c>
       <c r="D26">
-        <v>0.11</v>
+        <v>0.21</v>
       </c>
       <c r="E26">
-        <v>0.07</v>
+        <v>0.2</v>
       </c>
       <c r="F26">
+        <v>0.1773</v>
+      </c>
+      <c r="G26">
+        <v>0.1895</v>
+      </c>
+      <c r="H26">
         <v>0.2</v>
       </c>
-      <c r="G26">
-        <v>0.13</v>
-      </c>
-      <c r="H26">
-        <v>0.06</v>
-      </c>
       <c r="I26">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="J26">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -1202,31 +1202,31 @@
         <v>-喜歡</v>
       </c>
       <c r="B27">
-        <v>177</v>
+        <v>703</v>
       </c>
       <c r="C27">
-        <v>190</v>
+        <v>107</v>
       </c>
       <c r="D27">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E27">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="F27">
-        <v>132</v>
+        <v>43</v>
       </c>
       <c r="G27">
-        <v>145</v>
+        <v>83</v>
       </c>
       <c r="H27">
-        <v>158</v>
+        <v>138</v>
       </c>
       <c r="I27">
-        <v>171</v>
+        <v>67</v>
       </c>
       <c r="J27">
-        <v>184</v>
+        <v>53</v>
       </c>
       <c r="K27">
         <v>0</v>
@@ -1237,31 +1237,31 @@
         <v>-收藏</v>
       </c>
       <c r="B28">
-        <v>194</v>
+        <v>326</v>
       </c>
       <c r="C28">
-        <v>110</v>
+        <v>50</v>
       </c>
       <c r="D28">
-        <v>123</v>
+        <v>66</v>
       </c>
       <c r="E28">
-        <v>136</v>
+        <v>40</v>
       </c>
       <c r="F28">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="G28">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="H28">
-        <v>175</v>
+        <v>60</v>
       </c>
       <c r="I28">
-        <v>188</v>
+        <v>30</v>
       </c>
       <c r="J28">
-        <v>104</v>
+        <v>24</v>
       </c>
       <c r="K28">
         <v>0</v>
@@ -1272,31 +1272,31 @@
         <v>-分享</v>
       </c>
       <c r="B29">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="C29">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D29">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="E29">
-        <v>63</v>
+        <v>7</v>
       </c>
       <c r="F29">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="G29">
-        <v>89</v>
+        <v>12</v>
       </c>
       <c r="H29">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="I29">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="J29">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="K29">
         <v>0</v>
@@ -1312,34 +1312,34 @@
         <v>-發送篇數</v>
       </c>
       <c r="B31">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="C31">
         <v>0</v>
       </c>
       <c r="D31">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E31">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="H31">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="I31">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="J31">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="K31">
-        <v>78</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1347,34 +1347,34 @@
         <v>-關注人數</v>
       </c>
       <c r="B32">
-        <v>165</v>
+        <v>21</v>
       </c>
       <c r="C32">
         <v>0</v>
       </c>
       <c r="D32">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="E32">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="F32">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G32">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="H32">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="I32">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="J32">
-        <v>82</v>
+        <v>2</v>
       </c>
       <c r="K32">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -1382,34 +1382,34 @@
         <v>-閱讀量</v>
       </c>
       <c r="B33">
-        <v>182</v>
+        <v>583</v>
       </c>
       <c r="C33">
         <v>0</v>
       </c>
       <c r="D33">
-        <v>111</v>
+        <v>310</v>
       </c>
       <c r="E33">
-        <v>124</v>
+        <v>66</v>
       </c>
       <c r="F33">
         <v>0</v>
       </c>
       <c r="G33">
-        <v>150</v>
+        <v>55</v>
       </c>
       <c r="H33">
-        <v>163</v>
+        <v>105</v>
       </c>
       <c r="I33">
-        <v>176</v>
+        <v>25</v>
       </c>
       <c r="J33">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K33">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
@@ -1417,34 +1417,34 @@
         <v>-點讚</v>
       </c>
       <c r="B34">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C34">
         <v>0</v>
       </c>
       <c r="D34">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="E34">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="F34">
         <v>0</v>
       </c>
       <c r="G34">
-        <v>77</v>
+        <v>1</v>
       </c>
       <c r="H34">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I34">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="J34">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="K34">
-        <v>32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1452,34 +1452,34 @@
         <v>-推薦</v>
       </c>
       <c r="B35">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="C35">
         <v>0</v>
       </c>
       <c r="D35">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="E35">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="F35">
         <v>0</v>
       </c>
       <c r="G35">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H35">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I35">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="J35">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K35">
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1487,38 +1487,37 @@
         <v>-分享</v>
       </c>
       <c r="B36">
-        <v>136</v>
+        <v>29</v>
       </c>
       <c r="C36">
         <v>0</v>
       </c>
       <c r="D36">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E36">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="F36">
         <v>0</v>
       </c>
       <c r="G36">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H36">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="I36">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="J36">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="K36">
-        <v>66</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:N37"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Halve Xiaohongshu and WeChat figures and serve the test board on port 4187.
</commit_message>
<xml_diff>
--- a/public/samples/ctia-social-monthly.xlsx
+++ b/public/samples/ctia-social-monthly.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
@@ -452,34 +452,34 @@
         <v>-發送篇數</v>
       </c>
       <c r="B3">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
+        <v>7</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <v>6</v>
+      </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
+      <c r="J3">
+        <v>6</v>
+      </c>
+      <c r="K3">
         <v>2</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -487,34 +487,34 @@
         <v>-關注人數</v>
       </c>
       <c r="B4">
-        <v>155</v>
+        <v>393</v>
       </c>
       <c r="C4">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D4">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="E4">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="F4">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G4">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="H4">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="I4">
-        <v>34</v>
+        <v>86</v>
       </c>
       <c r="J4">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="K4">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -522,34 +522,34 @@
         <v>-閱讀/觀看量</v>
       </c>
       <c r="B5">
-        <v>8975</v>
+        <v>22445</v>
       </c>
       <c r="C5">
-        <v>404</v>
+        <v>1010</v>
       </c>
       <c r="D5">
-        <v>1285</v>
+        <v>3214</v>
       </c>
       <c r="E5">
-        <v>1580</v>
+        <v>3952</v>
       </c>
       <c r="F5">
-        <v>1449</v>
+        <v>3624</v>
       </c>
       <c r="G5">
-        <v>1695</v>
+        <v>4239</v>
       </c>
       <c r="H5">
-        <v>785</v>
+        <v>1964</v>
       </c>
       <c r="I5">
-        <v>1265</v>
+        <v>3163</v>
       </c>
       <c r="J5">
-        <v>478</v>
+        <v>1194</v>
       </c>
       <c r="K5">
-        <v>34</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6">
@@ -557,34 +557,34 @@
         <v>-喜歡/點讚量</v>
       </c>
       <c r="B6">
-        <v>1354</v>
+        <v>3395</v>
       </c>
       <c r="C6">
-        <v>115</v>
+        <v>289</v>
       </c>
       <c r="D6">
-        <v>129</v>
+        <v>324</v>
       </c>
       <c r="E6">
-        <v>325</v>
+        <v>816</v>
       </c>
       <c r="F6">
-        <v>47</v>
+        <v>118</v>
       </c>
       <c r="G6">
-        <v>93</v>
+        <v>232</v>
       </c>
       <c r="H6">
-        <v>190</v>
+        <v>476</v>
       </c>
       <c r="I6">
-        <v>248</v>
+        <v>621</v>
       </c>
       <c r="J6">
-        <v>194</v>
+        <v>486</v>
       </c>
       <c r="K6">
-        <v>13</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -592,34 +592,34 @@
         <v>-收藏/推薦量</v>
       </c>
       <c r="B7">
-        <v>599</v>
+        <v>1508</v>
       </c>
       <c r="C7">
-        <v>53</v>
+        <v>133</v>
       </c>
       <c r="D7">
-        <v>76</v>
+        <v>193</v>
       </c>
       <c r="E7">
-        <v>117</v>
+        <v>296</v>
       </c>
       <c r="F7">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G7">
-        <v>43</v>
+        <v>109</v>
       </c>
       <c r="H7">
-        <v>81</v>
+        <v>202</v>
       </c>
       <c r="I7">
-        <v>121</v>
+        <v>303</v>
       </c>
       <c r="J7">
-        <v>84</v>
+        <v>211</v>
       </c>
       <c r="K7">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -627,34 +627,34 @@
         <v>-分享量</v>
       </c>
       <c r="B8">
-        <v>160</v>
+        <v>405</v>
       </c>
       <c r="C8">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="D8">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="E8">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="F8">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="G8">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H8">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="I8">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="J8">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="K8">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -667,34 +667,34 @@
         <v>-曝光量</v>
       </c>
       <c r="B10">
-        <v>52707</v>
+        <v>131768</v>
       </c>
       <c r="C10">
-        <v>1965</v>
+        <v>4912</v>
       </c>
       <c r="D10">
-        <v>4777</v>
+        <v>11943</v>
       </c>
       <c r="E10">
-        <v>7455</v>
+        <v>18637</v>
       </c>
       <c r="F10">
-        <v>11479</v>
+        <v>28698</v>
       </c>
       <c r="G10">
-        <v>8091</v>
+        <v>20228</v>
       </c>
       <c r="H10">
-        <v>8360</v>
+        <v>20900</v>
       </c>
       <c r="I10">
-        <v>5900</v>
+        <v>14750</v>
       </c>
       <c r="J10">
-        <v>4560</v>
+        <v>11400</v>
       </c>
       <c r="K10">
-        <v>120</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11">
@@ -702,6 +702,7 @@
         <v>-點擊率</v>
       </c>
       <c r="B11">
+        <f>19%</f>
         <v>0.19</v>
       </c>
       <c r="C11">
@@ -742,34 +743,34 @@
         <v>-發送篇數</v>
       </c>
       <c r="B13">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>4</v>
+      </c>
+      <c r="J13">
+        <v>3</v>
+      </c>
+      <c r="K13">
         <v>1</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-      <c r="G13">
-        <v>1</v>
-      </c>
-      <c r="H13">
-        <v>1</v>
-      </c>
-      <c r="I13">
-        <v>2</v>
-      </c>
-      <c r="J13">
-        <v>1</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -777,34 +778,34 @@
         <v>-關注人數</v>
       </c>
       <c r="B14">
-        <v>57</v>
+        <v>143</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="I14">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="J14">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="K14">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -812,34 +813,34 @@
         <v>-曝光量</v>
       </c>
       <c r="B15">
-        <v>4436</v>
+        <v>11091</v>
       </c>
       <c r="C15">
-        <v>270</v>
+        <v>674</v>
       </c>
       <c r="D15">
-        <v>539</v>
+        <v>1349</v>
       </c>
       <c r="E15">
-        <v>674</v>
+        <v>1686</v>
       </c>
       <c r="F15">
-        <v>453</v>
+        <v>1132</v>
       </c>
       <c r="G15">
-        <v>480</v>
+        <v>1200</v>
       </c>
       <c r="H15">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="I15">
-        <v>900</v>
+        <v>2250</v>
       </c>
       <c r="J15">
-        <v>600</v>
+        <v>1500</v>
       </c>
       <c r="K15">
-        <v>120</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16">
@@ -847,34 +848,34 @@
         <v>-觀看量</v>
       </c>
       <c r="B16">
-        <v>1184</v>
+        <v>2959</v>
       </c>
       <c r="C16">
-        <v>67</v>
+        <v>168</v>
       </c>
       <c r="D16">
-        <v>134</v>
+        <v>335</v>
       </c>
       <c r="E16">
-        <v>168</v>
+        <v>419</v>
       </c>
       <c r="F16">
-        <v>169</v>
+        <v>422</v>
       </c>
       <c r="G16">
-        <v>136</v>
+        <v>340</v>
       </c>
       <c r="H16">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="I16">
-        <v>240</v>
+        <v>600</v>
       </c>
       <c r="J16">
-        <v>160</v>
+        <v>400</v>
       </c>
       <c r="K16">
-        <v>30</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17">
@@ -882,7 +883,7 @@
         <v>-點擊率</v>
       </c>
       <c r="B17">
-        <v>0.13336940348978762</v>
+        <v>0.13339644757010188</v>
       </c>
       <c r="C17">
         <v>0.14</v>
@@ -917,34 +918,34 @@
         <v>-喜歡</v>
       </c>
       <c r="B18">
-        <v>634</v>
+        <v>1589</v>
       </c>
       <c r="C18">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D18">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E18">
-        <v>215</v>
+        <v>540</v>
       </c>
       <c r="F18">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G18">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="H18">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="I18">
-        <v>180</v>
+        <v>450</v>
       </c>
       <c r="J18">
-        <v>140</v>
+        <v>350</v>
       </c>
       <c r="K18">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19">
@@ -952,34 +953,34 @@
         <v>-收藏</v>
       </c>
       <c r="B19">
-        <v>264</v>
+        <v>661</v>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D19">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E19">
-        <v>75</v>
+        <v>188</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="H19">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="I19">
-        <v>90</v>
+        <v>225</v>
       </c>
       <c r="J19">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="K19">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
@@ -987,34 +988,34 @@
         <v>-分享</v>
       </c>
       <c r="B20">
-        <v>53</v>
+        <v>131</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E20">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G20">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H20">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="I20">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J20">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="K20">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -1027,31 +1028,31 @@
         <v>-發送篇數</v>
       </c>
       <c r="B22">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E22">
+        <v>4</v>
+      </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
+      <c r="G22">
+        <v>3</v>
+      </c>
+      <c r="H22">
+        <v>3</v>
+      </c>
+      <c r="I22">
         <v>2</v>
       </c>
-      <c r="F22">
-        <v>1</v>
-      </c>
-      <c r="G22">
-        <v>1</v>
-      </c>
-      <c r="H22">
-        <v>1</v>
-      </c>
-      <c r="I22">
-        <v>1</v>
-      </c>
       <c r="J22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -1062,34 +1063,34 @@
         <v>-關注人數</v>
       </c>
       <c r="B23">
-        <v>77</v>
+        <v>195</v>
       </c>
       <c r="C23">
+        <v>35</v>
+      </c>
+      <c r="D23">
+        <v>40</v>
+      </c>
+      <c r="E23">
+        <v>45</v>
+      </c>
+      <c r="F23">
+        <v>20</v>
+      </c>
+      <c r="G23">
         <v>14</v>
       </c>
-      <c r="D23">
-        <v>16</v>
-      </c>
-      <c r="E23">
-        <v>18</v>
-      </c>
-      <c r="F23">
-        <v>8</v>
-      </c>
-      <c r="G23">
-        <v>5</v>
-      </c>
       <c r="H23">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="I23">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="J23">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K23">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -1097,31 +1098,31 @@
         <v>-曝光量</v>
       </c>
       <c r="B24">
-        <v>45348</v>
+        <v>113373</v>
       </c>
       <c r="C24">
-        <v>1695</v>
+        <v>4238</v>
       </c>
       <c r="D24">
-        <v>4238</v>
+        <v>10595</v>
       </c>
       <c r="E24">
-        <v>6780</v>
+        <v>16951</v>
       </c>
       <c r="F24">
-        <v>11026</v>
+        <v>27566</v>
       </c>
       <c r="G24">
-        <v>7609</v>
+        <v>19023</v>
       </c>
       <c r="H24">
-        <v>6000</v>
+        <v>15000</v>
       </c>
       <c r="I24">
-        <v>5000</v>
+        <v>12500</v>
       </c>
       <c r="J24">
-        <v>3000</v>
+        <v>7500</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -1132,31 +1133,31 @@
         <v>-觀看量</v>
       </c>
       <c r="B25">
-        <v>7211</v>
+        <v>18025</v>
       </c>
       <c r="C25">
-        <v>337</v>
+        <v>842</v>
       </c>
       <c r="D25">
-        <v>842</v>
+        <v>2104</v>
       </c>
       <c r="E25">
-        <v>1347</v>
+        <v>3367</v>
       </c>
       <c r="F25">
-        <v>1281</v>
+        <v>3202</v>
       </c>
       <c r="G25">
-        <v>1504</v>
+        <v>3760</v>
       </c>
       <c r="H25">
-        <v>600</v>
+        <v>1500</v>
       </c>
       <c r="I25">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="J25">
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -1167,7 +1168,7 @@
         <v>-點擊率</v>
       </c>
       <c r="B26">
-        <v>0.15898476261880085</v>
+        <v>0.15898847168197014</v>
       </c>
       <c r="C26">
         <v>0.22</v>
@@ -1202,31 +1203,31 @@
         <v>-喜歡</v>
       </c>
       <c r="B27">
-        <v>703</v>
+        <v>1757</v>
       </c>
       <c r="C27">
+        <v>269</v>
+      </c>
+      <c r="D27">
+        <v>259</v>
+      </c>
+      <c r="E27">
+        <v>269</v>
+      </c>
+      <c r="F27">
         <v>107</v>
       </c>
-      <c r="D27">
-        <v>104</v>
-      </c>
-      <c r="E27">
-        <v>108</v>
-      </c>
-      <c r="F27">
-        <v>43</v>
-      </c>
       <c r="G27">
-        <v>83</v>
+        <v>207</v>
       </c>
       <c r="H27">
-        <v>138</v>
+        <v>346</v>
       </c>
       <c r="I27">
-        <v>67</v>
+        <v>167</v>
       </c>
       <c r="J27">
-        <v>53</v>
+        <v>133</v>
       </c>
       <c r="K27">
         <v>0</v>
@@ -1237,31 +1238,31 @@
         <v>-收藏</v>
       </c>
       <c r="B28">
-        <v>326</v>
+        <v>820</v>
       </c>
       <c r="C28">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="D28">
-        <v>66</v>
+        <v>166</v>
       </c>
       <c r="E28">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="F28">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="G28">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="H28">
+        <v>150</v>
+      </c>
+      <c r="I28">
+        <v>75</v>
+      </c>
+      <c r="J28">
         <v>60</v>
-      </c>
-      <c r="I28">
-        <v>30</v>
-      </c>
-      <c r="J28">
-        <v>24</v>
       </c>
       <c r="K28">
         <v>0</v>
@@ -1272,31 +1273,31 @@
         <v>-分享</v>
       </c>
       <c r="B29">
-        <v>79</v>
+        <v>198</v>
       </c>
       <c r="C29">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D29">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E29">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="F29">
+        <v>38</v>
+      </c>
+      <c r="G29">
+        <v>29</v>
+      </c>
+      <c r="H29">
+        <v>40</v>
+      </c>
+      <c r="I29">
+        <v>20</v>
+      </c>
+      <c r="J29">
         <v>15</v>
-      </c>
-      <c r="G29">
-        <v>12</v>
-      </c>
-      <c r="H29">
-        <v>16</v>
-      </c>
-      <c r="I29">
-        <v>8</v>
-      </c>
-      <c r="J29">
-        <v>6</v>
       </c>
       <c r="K29">
         <v>0</v>
@@ -1312,34 +1313,34 @@
         <v>-發送篇數</v>
       </c>
       <c r="B31">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C31">
         <v>0</v>
       </c>
       <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31">
         <v>1</v>
       </c>
-      <c r="E31">
-        <v>0</v>
-      </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31">
+        <v>2</v>
+      </c>
+      <c r="H31">
         <v>1</v>
       </c>
-      <c r="H31">
-        <v>0</v>
-      </c>
       <c r="I31">
+        <v>2</v>
+      </c>
+      <c r="J31">
         <v>1</v>
       </c>
-      <c r="J31">
-        <v>0</v>
-      </c>
       <c r="K31">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1347,34 +1348,34 @@
         <v>-關注人數</v>
       </c>
       <c r="B32">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="C32">
         <v>0</v>
       </c>
       <c r="D32">
+        <v>13</v>
+      </c>
+      <c r="E32">
+        <v>8</v>
+      </c>
+      <c r="F32">
+        <v>3</v>
+      </c>
+      <c r="G32">
+        <v>7</v>
+      </c>
+      <c r="H32">
         <v>5</v>
       </c>
-      <c r="E32">
-        <v>3</v>
-      </c>
-      <c r="F32">
-        <v>1</v>
-      </c>
-      <c r="G32">
-        <v>3</v>
-      </c>
-      <c r="H32">
-        <v>2</v>
-      </c>
       <c r="I32">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J32">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K32">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -1382,34 +1383,34 @@
         <v>-閱讀量</v>
       </c>
       <c r="B33">
-        <v>583</v>
+        <v>1461</v>
       </c>
       <c r="C33">
         <v>0</v>
       </c>
       <c r="D33">
-        <v>310</v>
+        <v>775</v>
       </c>
       <c r="E33">
-        <v>66</v>
+        <v>166</v>
       </c>
       <c r="F33">
         <v>0</v>
       </c>
       <c r="G33">
-        <v>55</v>
+        <v>139</v>
       </c>
       <c r="H33">
-        <v>105</v>
+        <v>264</v>
       </c>
       <c r="I33">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="J33">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="K33">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34">
@@ -1417,34 +1418,34 @@
         <v>-點讚</v>
       </c>
       <c r="B34">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="C34">
         <v>0</v>
       </c>
       <c r="D34">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F34">
         <v>0</v>
       </c>
       <c r="G34">
+        <v>4</v>
+      </c>
+      <c r="H34">
+        <v>5</v>
+      </c>
+      <c r="I34">
+        <v>4</v>
+      </c>
+      <c r="J34">
+        <v>3</v>
+      </c>
+      <c r="K34">
         <v>1</v>
-      </c>
-      <c r="H34">
-        <v>2</v>
-      </c>
-      <c r="I34">
-        <v>1</v>
-      </c>
-      <c r="J34">
-        <v>1</v>
-      </c>
-      <c r="K34">
-        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1452,34 +1453,34 @@
         <v>-推薦</v>
       </c>
       <c r="B35">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="C35">
         <v>0</v>
       </c>
       <c r="D35">
+        <v>12</v>
+      </c>
+      <c r="E35">
         <v>5</v>
       </c>
-      <c r="E35">
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>3</v>
+      </c>
+      <c r="H35">
         <v>2</v>
       </c>
-      <c r="F35">
-        <v>0</v>
-      </c>
-      <c r="G35">
+      <c r="I35">
+        <v>3</v>
+      </c>
+      <c r="J35">
         <v>1</v>
       </c>
-      <c r="H35">
+      <c r="K35">
         <v>1</v>
-      </c>
-      <c r="I35">
-        <v>1</v>
-      </c>
-      <c r="J35">
-        <v>0</v>
-      </c>
-      <c r="K35">
-        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1487,37 +1488,38 @@
         <v>-分享</v>
       </c>
       <c r="B36">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="C36">
         <v>0</v>
       </c>
       <c r="D36">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="E36">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F36">
         <v>0</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H36">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I36">
+        <v>3</v>
+      </c>
+      <c r="J36">
+        <v>3</v>
+      </c>
+      <c r="K36">
         <v>1</v>
       </c>
-      <c r="J36">
-        <v>1</v>
-      </c>
-      <c r="K36">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:N37"/>
   </ignoredErrors>

</xml_diff>